<commit_message>
Remove Farglory specific reports from analysis tracking tables
</commit_message>
<xml_diff>
--- a/All_Reports_Scraping_Analysis.xlsx
+++ b/All_Reports_Scraping_Analysis.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Australia_27份" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="London_28份" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Australia_Filtered" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="London_Filtered" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,51 +605,24 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2505 Australia_Prepared for Farglory LaSalle.pdf</t>
+          <t>20250701_RCA_Transaction_Report $100m+ 2024-present.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.lasalle.com/research</t>
+          <t>https://www.msci.com/our-solutions/real-assets/real-capital-analytics</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>⚠️ 阻擋且網頁改版 (404)</t>
+          <t>✅ 可通行 (可能需登入)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
-        <is>
-          <t>1. 需先繞過防火牆
-2. 找出新版報告網址
-3. 實作下載邏輯</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>20250701_RCA_Transaction_Report $100m+ 2024-present.pdf</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://www.msci.com/our-solutions/real-assets/real-capital-analytics</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>✅ 可通行 (可能需登入)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
         <is>
           <t>1. 存取 MSCI 平台頁面
 2. 若報告為付費牆內，實作自動登入
@@ -657,18 +630,43 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JLL apac property investment guide 2024.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.jll.com.au/en/trends-and-insights/research</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>✅ 可通行 (200)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(同編號 1，屬 JLL 操作流程，需處理填表邏輯)</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JLL apac property investment guide 2024.pdf</t>
+          <t>KWM-Investing-Down-Under-Guide-2025.pdf</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.jll.com.au/en/trends-and-insights/research</t>
+          <t>https://www.kwm.com/au/en/insights.html</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -678,74 +676,74 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(同編號 1，屬 JLL 操作流程，需處理填表邏輯)</t>
+          <t>1. 存取 KWM 洞察專區
+2. 尋找 PDF 標籤下載</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KWM-Investing-Down-Under-Guide-2025.pdf</t>
+          <t>Sydney and Brisbane office markets.docx</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.kwm.com/au/en/insights.html</t>
+          <t>(未具名/待確認來源)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>✅ 可通行 (200)</t>
+          <t>❓ 來源不明</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1. 存取 KWM 洞察專區
-2. 尋找 PDF 標籤下載</t>
+          <t>1. 需客戶確認發布機構官網
+2. 工程師評估抓取方式</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sydney and Brisbane office markets.docx</t>
+          <t>24Q4 brisbane-office-market-dynamic_JLL.pdf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>(未具名/待確認來源)</t>
+          <t>https://www.jll.com.au/en/trends-and-insights/research</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>❓ 來源不明</t>
+          <t>✅ 可通行 (200)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1. 需客戶確認發布機構官網
-2. 工程師評估抓取方式</t>
+          <t>(同編號 1，屬 JLL 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>24Q4 brisbane-office-market-dynamic_JLL.pdf</t>
+          <t>24Q4_Research_Figures_-_Brisbane_ CBRE.pdf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.jll.com.au/en/trends-and-insights/research</t>
+          <t>https://www.cbre.com.au/insights</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -755,22 +753,23 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(同編號 1，屬 JLL 操作流程)</t>
+          <t>1. 存取 CBRE 頁面
+2. 模擬填寫表單或直接抓取 PDF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>24Q4_Research_Figures_-_Brisbane_ CBRE.pdf</t>
+          <t>25Q1 brisbane-cbd-office-state-of-the-market-KF.pdf</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.cbre.com.au/insights</t>
+          <t>https://www.knightfrank.com.au/research</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -780,23 +779,23 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1. 存取 CBRE 頁面
-2. 模擬填寫表單或直接抓取 PDF</t>
+          <t>1. 存取萊坊研究專區
+2. 下載 PDF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25Q1 brisbane-cbd-office-state-of-the-market-KF.pdf</t>
+          <t>25Q1_Research_Figures_-_Brisbane- CBRE.pdf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.knightfrank.com.au/research</t>
+          <t>https://www.cbre.com.au/insights</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -806,73 +805,72 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1. 存取萊坊研究專區
-2. 下載 PDF</t>
+          <t>(同編號 13，屬 CBRE 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25Q1_Research_Figures_-_Brisbane- CBRE.pdf</t>
+          <t>2405 Into the Golden Decade..._Colliers.pdf</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.cbre.com.au/insights</t>
+          <t>https://www.colliers.com.au/en-au/research</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>✅ 可通行 (200)</t>
+          <t>🛡️ 有防護 (需繞過 Cloudflare)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>(同編號 13，屬 CBRE 操作流程)</t>
+          <t>(同編號 3，屬 Colliers 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2405 Into the Golden Decade..._Colliers.pdf</t>
+          <t>2504- brisbane-cbd-office-market-KF.pdf</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.colliers.com.au/en-au/research</t>
+          <t>https://www.knightfrank.com.au/research</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>🛡️ 有防護 (需繞過 Cloudflare)</t>
+          <t>✅ 可通行 (200)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(同編號 3，屬 Colliers 操作流程)</t>
+          <t>(同編號 14，屬萊坊操作流程)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2504- brisbane-cbd-office-market-KF.pdf</t>
+          <t>Olympics Brisbane_CBRE.pdf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.knightfrank.com.au/research</t>
+          <t>https://www.cbre.com.au/insights</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -882,93 +880,93 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(同編號 14，屬萊坊操作流程)</t>
+          <t>(同編號 13，屬 CBRE 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Olympics Brisbane_CBRE.pdf</t>
+          <t>24H2-syd-Savills.pdf</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.cbre.com.au/insights</t>
+          <t>https://www.savills.com.au/research.aspx</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>✅ 可通行 (200)</t>
+          <t>⚠️ 網頁失效/改版 (404)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(同編號 13，屬 CBRE 操作流程)</t>
+          <t>1. 至 Savills 官網尋找新網址
+2. 撰寫下載流程</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>24H2-syd-Savills.pdf</t>
+          <t>24Q4 CBD Office Snapshot-Colliers.pdf</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.savills.com.au/research.aspx</t>
+          <t>https://www.colliers.com.au/en-au/research</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>⚠️ 網頁失效/改版 (404)</t>
+          <t>🛡️ 有防護 (需繞過 Cloudflare)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1. 至 Savills 官網尋找新網址
-2. 撰寫下載流程</t>
+          <t>(同編號 3，屬 Colliers 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>24Q4 CBD Office Snapshot-Colliers.pdf</t>
+          <t>24Q4_Research_Figures_-_Sydney_CBRE.pdf</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.colliers.com.au/en-au/research</t>
+          <t>https://www.cbre.com.au/insights</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>🛡️ 有防護 (需繞過 Cloudflare)</t>
+          <t>✅ 可通行 (200)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(同編號 3，屬 Colliers 操作流程)</t>
+          <t>(同編號 13，屬 CBRE 操作流程)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>24Q4_Research_Figures_-_Sydney_CBRE.pdf</t>
+          <t>25Q1_Research_Figures_-_Sydney-CBRE.pdf</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -989,16 +987,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25Q1_Research_Figures_-_Sydney-CBRE.pdf</t>
+          <t>25Q1-sydney-cbd-office_Cushman.pdf</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.cbre.com.au/insights</t>
+          <t>https://www.cushmanwakefield.com/en/australia/insights</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1008,22 +1006,23 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(同編號 13，屬 CBRE 操作流程)</t>
+          <t>1. 存取戴德梁行 Insights 專區
+2. 解析下載點</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25Q1-sydney-cbd-office_Cushman.pdf</t>
+          <t>25Q1-sydney-cbd-office-state- KF.pdf</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.cushmanwakefield.com/en/australia/insights</t>
+          <t>https://www.knightfrank.com.au/research</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1033,23 +1032,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1. 存取戴德梁行 Insights 專區
-2. 解析下載點</t>
+          <t>(同編號 14，屬萊坊操作流程)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25Q1-sydney-cbd-office-state- KF.pdf</t>
+          <t>2501 Office market report propoertycouncil.pdf</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.knightfrank.com.au/research</t>
+          <t>https://www.propertycouncil.com.au/research</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1059,22 +1057,23 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>(同編號 14，屬萊坊操作流程)</t>
+          <t>1. 存取澳洲地產委員會專區
+2. 解析報告列表</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2501 Office market report propoertycouncil.pdf</t>
+          <t>2502 sydney-cbd-office-market KF.pdf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.propertycouncil.com.au/research</t>
+          <t>https://www.knightfrank.com.au/research</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1084,18 +1083,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1. 存取澳洲地產委員會專區
-2. 解析報告列表</t>
+          <t>(同編號 14，屬萊坊操作流程)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2502 sydney-cbd-office-market KF.pdf</t>
+          <t>Map CBD 18 sydney-cbd-office-market KF.pdf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1109,31 +1107,6 @@
         </is>
       </c>
       <c r="E27" t="inlineStr">
-        <is>
-          <t>(同編號 14，屬萊坊操作流程)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Map CBD 18 sydney-cbd-office-market KF.pdf</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>https://www.knightfrank.com.au/research</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>✅ 可通行 (200)</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
         <is>
           <t>(同編號 14，屬萊坊操作流程)</t>
         </is>
@@ -1150,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1770,88 +1743,87 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Q2 2024 Central London Office Market - Farglory.pdf</t>
+          <t>Q3 2024 Central London Office Market -Quadrant.pdf</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>(Farglory 客製化報告)</t>
+          <t>https://www.quadrantestates.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>❓ 需提供管道</t>
+          <t>⚠️ 確切研報網址需更新 (404)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1. 建議不寫網頁爬蟲
-2. 改寫 E-mail 自動收信腳本</t>
+          <t>(同編號 6)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Q3 2024 Central London Office Market -Quadrant.pdf</t>
+          <t>September 2024 - Brief Market Update.pdf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.quadrantestates.com/</t>
+          <t>(未具名短報)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>⚠️ 確切研報網址需更新 (404)</t>
+          <t>❓ 需確認來源</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>(同編號 6)</t>
+          <t>1. 確認發行單位
+2. 套用該單位的邏輯</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>September 2024 - Brief Market Update.pdf</t>
+          <t>west-end-investment-watch-aug-24.pdf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>(未具名短報)</t>
+          <t>https://www.savills.co.uk/insight-and-opinion/research.aspx</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>❓ 需確認來源</t>
+          <t>⚠️ 網頁改版/需更新 URL (404)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1. 確認發行單位
-2. 套用該單位的邏輯</t>
+          <t>(同編號 7)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>west-end-investment-watch-aug-24.pdf</t>
+          <t>West-End-Investment-Watch-Sep-24.pdf</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1865,31 +1837,6 @@
         </is>
       </c>
       <c r="E28" t="inlineStr">
-        <is>
-          <t>(同編號 7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>West-End-Investment-Watch-Sep-24.pdf</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>https://www.savills.co.uk/insight-and-opinion/research.aspx</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>⚠️ 網頁改版/需更新 URL (404)</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
         <is>
           <t>(同編號 7)</t>
         </is>

</xml_diff>